<commit_message>
Selesai untuk phase ini. - Semua form CRUD kini mendapat feedback Fomantic UI di dalam form: status sukses, ringkasan error, dan penandaan field bermasalah, selain toast global. - Upload foto profil diperbaiki dengan validasi JPG/PNG/WebP maksimal 3 MB, live preview, cache busting, pembaruan avatar, dan penghapusan foto lama. - Periode anggaran dibatasi:   - Role daerah memakai rentang RPJMD.   - Role OPD hanya memakai Renstra OPD terkait.   - Tahun hanya dapat dipilih dalam rentang aktif.   - Validasi server mencegah manipulasi periode dari request manual. - Excel Renja/RKA/DPA dan perubahannya memiliki:   - Satu sheet per subkegiatan.   - Metadata dokumen.   - Hierarki kode rekening dan uraian.   - Kolom volume, satuan, harga, PPN, jumlah, sebelum/sesudah, dan selisih.   - Total DPPA telah dikoreksi agar berada tepat pada kolom Jumlah G dan L.   - Warna, border, orientasi, freeze pane, dan lebar kolom resmi.
</commit_message>
<xml_diff>
--- a/outputs/01a058f3-6239-7122-bdb7-1ec257ed0d1d/dppa-format-resmi.xlsx
+++ b/outputs/01a058f3-6239-7122-bdb7-1ec257ed0d1d/dppa-format-resmi.xlsx
@@ -1012,20 +1012,20 @@
         <v>33</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="12">
-        <v>75000000.0</v>
-      </c>
+      <c r="C19" s="12"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12">
-        <v>103000000.0</v>
-      </c>
+      <c r="G19" s="12">
+        <v>75000000.0</v>
+      </c>
+      <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12">
+        <v>103000000.0</v>
+      </c>
       <c r="M19" s="12">
         <v>28000000.0</v>
       </c>
@@ -1471,20 +1471,20 @@
         <v>33</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="12">
-        <v>75000000.0</v>
-      </c>
+      <c r="C19" s="12"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12">
-        <v>104000000.0</v>
-      </c>
+      <c r="G19" s="12">
+        <v>75000000.0</v>
+      </c>
+      <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12">
+        <v>104000000.0</v>
+      </c>
       <c r="M19" s="12">
         <v>29000000.0</v>
       </c>
@@ -1930,20 +1930,20 @@
         <v>33</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="12">
-        <v>75000000.0</v>
-      </c>
+      <c r="C19" s="12"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12">
-        <v>105000000.0</v>
-      </c>
+      <c r="G19" s="12">
+        <v>75000000.0</v>
+      </c>
+      <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12">
+        <v>105000000.0</v>
+      </c>
       <c r="M19" s="12">
         <v>30000000.0</v>
       </c>
@@ -2416,20 +2416,20 @@
         <v>33</v>
       </c>
       <c r="B20" s="8"/>
-      <c r="C20" s="12">
-        <v>315000000.0</v>
-      </c>
+      <c r="C20" s="12"/>
       <c r="D20" s="12"/>
       <c r="E20" s="12"/>
       <c r="F20" s="16"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12">
-        <v>332500000.0</v>
-      </c>
+      <c r="G20" s="12">
+        <v>315000000.0</v>
+      </c>
+      <c r="H20" s="12"/>
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
+      <c r="L20" s="12">
+        <v>332500000.0</v>
+      </c>
       <c r="M20" s="12">
         <v>17500000.0</v>
       </c>
@@ -2867,20 +2867,20 @@
         <v>33</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="12">
-        <v>180000000.0</v>
-      </c>
+      <c r="C19" s="12"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12">
-        <v>190000000.0</v>
-      </c>
+      <c r="G19" s="12">
+        <v>180000000.0</v>
+      </c>
+      <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12">
+        <v>190000000.0</v>
+      </c>
       <c r="M19" s="12">
         <v>10000000.0</v>
       </c>

</xml_diff>